<commit_message>
upload my day 04 excel using pivote table
</commit_message>
<xml_diff>
--- a/excel-files/day - 03 Lookups.xlsx
+++ b/excel-files/day - 03 Lookups.xlsx
@@ -2,22 +2,26 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr defaultThemeVersion="166925"/>
+  <workbookPr hidePivotFieldList="1" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/12a4f0da8943f55f/Data Science Journey/healthcare-analyst-journey/Excel Files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="107" documentId="8_{A6ECC9B9-9FE0-46C9-93ED-84AC59A511E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{671011E9-BE30-4DBD-B859-901949F57DF3}"/>
+  <xr:revisionPtr revIDLastSave="224" documentId="8_{A6ECC9B9-9FE0-46C9-93ED-84AC59A511E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E5F964E1-FFCD-4B1B-9495-29A2982DD7FC}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{04C2A604-B662-4EF3-9182-2D379372EE84}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{04C2A604-B662-4EF3-9182-2D379372EE84}"/>
   </bookViews>
   <sheets>
     <sheet name="Patient_records" sheetId="1" r:id="rId1"/>
     <sheet name="Department_info" sheetId="2" r:id="rId2"/>
+    <sheet name="Pivot_reports" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
+  <pivotCaches>
+    <pivotCache cacheId="43" r:id="rId4"/>
+    <pivotCache cacheId="47" r:id="rId5"/>
+  </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -41,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="127">
   <si>
     <t>Age</t>
   </si>
@@ -386,6 +390,42 @@
   </si>
   <si>
     <t xml:space="preserve">Bed Occupency </t>
+  </si>
+  <si>
+    <t>Grand Total</t>
+  </si>
+  <si>
+    <t>Count of Patient ID</t>
+  </si>
+  <si>
+    <t>(All)</t>
+  </si>
+  <si>
+    <t>Apr</t>
+  </si>
+  <si>
+    <t>May</t>
+  </si>
+  <si>
+    <t>Column Labels</t>
+  </si>
+  <si>
+    <t>Departments</t>
+  </si>
+  <si>
+    <t>Average of Age</t>
+  </si>
+  <si>
+    <t>Months</t>
+  </si>
+  <si>
+    <t>city</t>
+  </si>
+  <si>
+    <t>Senior category</t>
+  </si>
+  <si>
+    <t>Count of Senior category</t>
   </si>
 </sst>
 </file>
@@ -393,7 +433,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="175" formatCode="0.0"/>
+    <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -469,7 +509,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -482,13 +522,249 @@
     <xf numFmtId="9" fontId="3" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="175" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="76">
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="171" formatCode="0.000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="171" formatCode="0.000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="170" formatCode="0.0000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="170" formatCode="0.0000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="169" formatCode="0.00000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="169" formatCode="0.00000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="0.000000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="0.000000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="0.0000000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="0.0000000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.00000000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.00000000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="0.000000000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="0.000000000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.00000000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.00000000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="0.0000000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="0.0000000"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -499,6 +775,2393 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
+<file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Praveen Tirumani" refreshedDate="46145.476931944446" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="30" xr:uid="{A3E0F538-46EE-4982-96FF-AA43AE62C081}">
+  <cacheSource type="worksheet">
+    <worksheetSource ref="A1:K31" sheet="Patient_records"/>
+  </cacheSource>
+  <cacheFields count="12">
+    <cacheField name="Patient ID" numFmtId="0">
+      <sharedItems count="30">
+        <s v="A10001"/>
+        <s v="A10002"/>
+        <s v="A10003"/>
+        <s v="A10004"/>
+        <s v="A10005"/>
+        <s v="A10006"/>
+        <s v="A10007"/>
+        <s v="A10008"/>
+        <s v="A10009"/>
+        <s v="A10010"/>
+        <s v="A10011"/>
+        <s v="A10012"/>
+        <s v="A10013"/>
+        <s v="A10014"/>
+        <s v="A10015"/>
+        <s v="A10016"/>
+        <s v="A10017"/>
+        <s v="A10018"/>
+        <s v="A10019"/>
+        <s v="A10020"/>
+        <s v="A10021"/>
+        <s v="A10022"/>
+        <s v="A10023"/>
+        <s v="A10024"/>
+        <s v="A10025"/>
+        <s v="A10026"/>
+        <s v="A10027"/>
+        <s v="A10028"/>
+        <s v="A10029"/>
+        <s v="A10030"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Name " numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Age" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="18" maxValue="45"/>
+    </cacheField>
+    <cacheField name="Gender" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="City" numFmtId="0">
+      <sharedItems count="19">
+        <s v="Hyderabad"/>
+        <s v="Gudivada"/>
+        <s v="Begumpet"/>
+        <s v="Amaravathi"/>
+        <s v="Godavari"/>
+        <s v="Konaseema"/>
+        <s v="Malakpet"/>
+        <s v="Kondaput"/>
+        <s v="Hafeezpet"/>
+        <s v="High tech city"/>
+        <s v="Kondapur"/>
+        <s v="Nandigama"/>
+        <s v="Singareni"/>
+        <s v="Rajkot"/>
+        <s v="Bengalore"/>
+        <s v="Vizag"/>
+        <s v="Petrorius"/>
+        <s v="Nalgonda"/>
+        <s v="Chennai"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Appointment Date" numFmtId="14">
+      <sharedItems containsSemiMixedTypes="0" containsNonDate="0" containsDate="1" containsString="0" minDate="2026-04-30T00:00:00" maxDate="2026-05-30T00:00:00" count="30">
+        <d v="2026-04-30T00:00:00"/>
+        <d v="2026-05-01T00:00:00"/>
+        <d v="2026-05-02T00:00:00"/>
+        <d v="2026-05-03T00:00:00"/>
+        <d v="2026-05-04T00:00:00"/>
+        <d v="2026-05-05T00:00:00"/>
+        <d v="2026-05-06T00:00:00"/>
+        <d v="2026-05-07T00:00:00"/>
+        <d v="2026-05-08T00:00:00"/>
+        <d v="2026-05-09T00:00:00"/>
+        <d v="2026-05-10T00:00:00"/>
+        <d v="2026-05-11T00:00:00"/>
+        <d v="2026-05-12T00:00:00"/>
+        <d v="2026-05-13T00:00:00"/>
+        <d v="2026-05-14T00:00:00"/>
+        <d v="2026-05-15T00:00:00"/>
+        <d v="2026-05-16T00:00:00"/>
+        <d v="2026-05-17T00:00:00"/>
+        <d v="2026-05-18T00:00:00"/>
+        <d v="2026-05-19T00:00:00"/>
+        <d v="2026-05-20T00:00:00"/>
+        <d v="2026-05-21T00:00:00"/>
+        <d v="2026-05-22T00:00:00"/>
+        <d v="2026-05-23T00:00:00"/>
+        <d v="2026-05-24T00:00:00"/>
+        <d v="2026-05-25T00:00:00"/>
+        <d v="2026-05-26T00:00:00"/>
+        <d v="2026-05-27T00:00:00"/>
+        <d v="2026-05-28T00:00:00"/>
+        <d v="2026-05-29T00:00:00"/>
+      </sharedItems>
+      <fieldGroup par="11"/>
+    </cacheField>
+    <cacheField name="Dapartment Name" numFmtId="0">
+      <sharedItems count="5">
+        <s v="Cardiology"/>
+        <s v="Emergency"/>
+        <s v="Neurology"/>
+        <s v="Pediatrics"/>
+        <s v="Orthopedics"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Showed Up" numFmtId="0">
+      <sharedItems count="2">
+        <s v="Yes"/>
+        <s v="No"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Department ID" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Head Doctor" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Bed Capacity" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="35" maxValue="70"/>
+    </cacheField>
+    <cacheField name="Months (Appointment Date)" numFmtId="0" databaseField="0">
+      <fieldGroup base="5">
+        <rangePr groupBy="months" startDate="2026-04-30T00:00:00" endDate="2026-05-30T00:00:00"/>
+        <groupItems count="14">
+          <s v="&lt;30-04-2026"/>
+          <s v="Jan"/>
+          <s v="Feb"/>
+          <s v="Mar"/>
+          <s v="Apr"/>
+          <s v="May"/>
+          <s v="Jun"/>
+          <s v="Jul"/>
+          <s v="Aug"/>
+          <s v="Sep"/>
+          <s v="Oct"/>
+          <s v="Nov"/>
+          <s v="Dec"/>
+          <s v="&gt;30-05-2026"/>
+        </groupItems>
+      </fieldGroup>
+    </cacheField>
+  </cacheFields>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl/pivotCache/pivotCacheDefinition2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Praveen Tirumani" refreshedDate="46145.477733564818" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="30" xr:uid="{2CA04E71-E486-45DD-90BB-36D1799F6065}">
+  <cacheSource type="worksheet">
+    <worksheetSource ref="A1:L31" sheet="Patient_records"/>
+  </cacheSource>
+  <cacheFields count="12">
+    <cacheField name="Patient ID" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Name " numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Age" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="18" maxValue="45"/>
+    </cacheField>
+    <cacheField name="Gender" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="City" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Appointment Date" numFmtId="14">
+      <sharedItems containsSemiMixedTypes="0" containsNonDate="0" containsDate="1" containsString="0" minDate="2026-04-30T00:00:00" maxDate="2026-05-30T00:00:00"/>
+    </cacheField>
+    <cacheField name="Dapartment Name" numFmtId="0">
+      <sharedItems count="5">
+        <s v="Cardiology"/>
+        <s v="Emergency"/>
+        <s v="Neurology"/>
+        <s v="Pediatrics"/>
+        <s v="Orthopedics"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Showed Up" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Department ID" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Head Doctor" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Bed Capacity" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="35" maxValue="70"/>
+    </cacheField>
+    <cacheField name="Senior category" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+  </cacheFields>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="30">
+  <r>
+    <x v="0"/>
+    <s v="Praveen"/>
+    <n v="28"/>
+    <s v="Male"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <s v="D001"/>
+    <s v="Dr. Rao"/>
+    <n v="50"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <s v="Dhanush"/>
+    <n v="22"/>
+    <s v="Male"/>
+    <x v="0"/>
+    <x v="1"/>
+    <x v="1"/>
+    <x v="0"/>
+    <s v="D005"/>
+    <s v="Dr. Reddy"/>
+    <n v="70"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <s v="Harpreet"/>
+    <n v="22"/>
+    <s v="Male"/>
+    <x v="0"/>
+    <x v="2"/>
+    <x v="2"/>
+    <x v="1"/>
+    <s v="D002"/>
+    <s v="Dr. Mehta"/>
+    <n v="40"/>
+  </r>
+  <r>
+    <x v="3"/>
+    <s v="Sekhar"/>
+    <n v="19"/>
+    <s v="Male"/>
+    <x v="0"/>
+    <x v="3"/>
+    <x v="3"/>
+    <x v="1"/>
+    <s v="D004"/>
+    <s v="Dr. Sharma"/>
+    <n v="35"/>
+  </r>
+  <r>
+    <x v="4"/>
+    <s v="Rangayya"/>
+    <n v="20"/>
+    <s v="Male"/>
+    <x v="1"/>
+    <x v="4"/>
+    <x v="4"/>
+    <x v="0"/>
+    <s v="D003"/>
+    <s v="Dr. Kumar"/>
+    <n v="60"/>
+  </r>
+  <r>
+    <x v="5"/>
+    <s v="Rangamma"/>
+    <n v="18"/>
+    <s v="Female"/>
+    <x v="1"/>
+    <x v="5"/>
+    <x v="0"/>
+    <x v="0"/>
+    <s v="D001"/>
+    <s v="Dr. Rao"/>
+    <n v="50"/>
+  </r>
+  <r>
+    <x v="6"/>
+    <s v="Mogalayya"/>
+    <n v="25"/>
+    <s v="Male"/>
+    <x v="2"/>
+    <x v="6"/>
+    <x v="2"/>
+    <x v="0"/>
+    <s v="D002"/>
+    <s v="Dr. Mehta"/>
+    <n v="40"/>
+  </r>
+  <r>
+    <x v="7"/>
+    <s v="Jangayya"/>
+    <n v="45"/>
+    <s v="Male"/>
+    <x v="3"/>
+    <x v="7"/>
+    <x v="0"/>
+    <x v="0"/>
+    <s v="D001"/>
+    <s v="Dr. Rao"/>
+    <n v="50"/>
+  </r>
+  <r>
+    <x v="8"/>
+    <s v="Madhu"/>
+    <n v="22"/>
+    <s v="Male"/>
+    <x v="4"/>
+    <x v="8"/>
+    <x v="1"/>
+    <x v="0"/>
+    <s v="D005"/>
+    <s v="Dr. Reddy"/>
+    <n v="70"/>
+  </r>
+  <r>
+    <x v="9"/>
+    <s v="Rudra"/>
+    <n v="28"/>
+    <s v="Male"/>
+    <x v="5"/>
+    <x v="9"/>
+    <x v="2"/>
+    <x v="0"/>
+    <s v="D002"/>
+    <s v="Dr. Mehta"/>
+    <n v="40"/>
+  </r>
+  <r>
+    <x v="10"/>
+    <s v="Mehar"/>
+    <n v="29"/>
+    <s v="Female"/>
+    <x v="6"/>
+    <x v="10"/>
+    <x v="3"/>
+    <x v="0"/>
+    <s v="D004"/>
+    <s v="Dr. Sharma"/>
+    <n v="35"/>
+  </r>
+  <r>
+    <x v="11"/>
+    <s v="mohan"/>
+    <n v="34"/>
+    <s v="Male"/>
+    <x v="7"/>
+    <x v="11"/>
+    <x v="4"/>
+    <x v="0"/>
+    <s v="D003"/>
+    <s v="Dr. Kumar"/>
+    <n v="60"/>
+  </r>
+  <r>
+    <x v="12"/>
+    <s v="Radhika"/>
+    <n v="22"/>
+    <s v="Female"/>
+    <x v="8"/>
+    <x v="12"/>
+    <x v="0"/>
+    <x v="0"/>
+    <s v="D001"/>
+    <s v="Dr. Rao"/>
+    <n v="50"/>
+  </r>
+  <r>
+    <x v="13"/>
+    <s v="Mounika"/>
+    <n v="30"/>
+    <s v="Female"/>
+    <x v="9"/>
+    <x v="13"/>
+    <x v="2"/>
+    <x v="0"/>
+    <s v="D002"/>
+    <s v="Dr. Mehta"/>
+    <n v="40"/>
+  </r>
+  <r>
+    <x v="14"/>
+    <s v="Meghana"/>
+    <n v="20"/>
+    <s v="Female"/>
+    <x v="10"/>
+    <x v="14"/>
+    <x v="0"/>
+    <x v="1"/>
+    <s v="D001"/>
+    <s v="Dr. Rao"/>
+    <n v="50"/>
+  </r>
+  <r>
+    <x v="15"/>
+    <s v="Nagalaxmi"/>
+    <n v="20"/>
+    <s v="Female"/>
+    <x v="11"/>
+    <x v="15"/>
+    <x v="1"/>
+    <x v="0"/>
+    <s v="D005"/>
+    <s v="Dr. Reddy"/>
+    <n v="70"/>
+  </r>
+  <r>
+    <x v="16"/>
+    <s v="Manoj"/>
+    <n v="29"/>
+    <s v="Male"/>
+    <x v="11"/>
+    <x v="16"/>
+    <x v="2"/>
+    <x v="1"/>
+    <s v="D002"/>
+    <s v="Dr. Mehta"/>
+    <n v="40"/>
+  </r>
+  <r>
+    <x v="17"/>
+    <s v="Rekha"/>
+    <n v="29"/>
+    <s v="Female"/>
+    <x v="10"/>
+    <x v="17"/>
+    <x v="3"/>
+    <x v="1"/>
+    <s v="D004"/>
+    <s v="Dr. Sharma"/>
+    <n v="35"/>
+  </r>
+  <r>
+    <x v="18"/>
+    <s v="Happie"/>
+    <n v="20"/>
+    <s v="Female"/>
+    <x v="6"/>
+    <x v="18"/>
+    <x v="4"/>
+    <x v="0"/>
+    <s v="D003"/>
+    <s v="Dr. Kumar"/>
+    <n v="60"/>
+  </r>
+  <r>
+    <x v="19"/>
+    <s v="Nagarjuna"/>
+    <n v="29"/>
+    <s v="Male"/>
+    <x v="12"/>
+    <x v="19"/>
+    <x v="0"/>
+    <x v="1"/>
+    <s v="D001"/>
+    <s v="Dr. Rao"/>
+    <n v="50"/>
+  </r>
+  <r>
+    <x v="20"/>
+    <s v="Sikhar"/>
+    <n v="28"/>
+    <s v="Male"/>
+    <x v="13"/>
+    <x v="20"/>
+    <x v="2"/>
+    <x v="0"/>
+    <s v="D002"/>
+    <s v="Dr. Mehta"/>
+    <n v="40"/>
+  </r>
+  <r>
+    <x v="21"/>
+    <s v="Dhawan"/>
+    <n v="45"/>
+    <s v="Male"/>
+    <x v="14"/>
+    <x v="21"/>
+    <x v="0"/>
+    <x v="0"/>
+    <s v="D001"/>
+    <s v="Dr. Rao"/>
+    <n v="50"/>
+  </r>
+  <r>
+    <x v="22"/>
+    <s v="Neelambari"/>
+    <n v="34"/>
+    <s v="Female"/>
+    <x v="0"/>
+    <x v="22"/>
+    <x v="1"/>
+    <x v="0"/>
+    <s v="D005"/>
+    <s v="Dr. Reddy"/>
+    <n v="70"/>
+  </r>
+  <r>
+    <x v="23"/>
+    <s v="Aravind"/>
+    <n v="22"/>
+    <s v="Male"/>
+    <x v="0"/>
+    <x v="23"/>
+    <x v="2"/>
+    <x v="1"/>
+    <s v="D002"/>
+    <s v="Dr. Mehta"/>
+    <n v="40"/>
+  </r>
+  <r>
+    <x v="24"/>
+    <s v="Meghana"/>
+    <n v="24"/>
+    <s v="Female"/>
+    <x v="0"/>
+    <x v="24"/>
+    <x v="3"/>
+    <x v="1"/>
+    <s v="D004"/>
+    <s v="Dr. Sharma"/>
+    <n v="35"/>
+  </r>
+  <r>
+    <x v="25"/>
+    <s v="Simha"/>
+    <n v="34"/>
+    <s v="Male"/>
+    <x v="4"/>
+    <x v="25"/>
+    <x v="4"/>
+    <x v="0"/>
+    <s v="D003"/>
+    <s v="Dr. Kumar"/>
+    <n v="60"/>
+  </r>
+  <r>
+    <x v="26"/>
+    <s v="Reddy"/>
+    <n v="23"/>
+    <s v="Male"/>
+    <x v="15"/>
+    <x v="26"/>
+    <x v="0"/>
+    <x v="0"/>
+    <s v="D001"/>
+    <s v="Dr. Rao"/>
+    <n v="50"/>
+  </r>
+  <r>
+    <x v="27"/>
+    <s v="Klassen"/>
+    <n v="34"/>
+    <s v="Male"/>
+    <x v="16"/>
+    <x v="27"/>
+    <x v="2"/>
+    <x v="0"/>
+    <s v="D002"/>
+    <s v="Dr. Mehta"/>
+    <n v="40"/>
+  </r>
+  <r>
+    <x v="28"/>
+    <s v="Mouna"/>
+    <n v="28"/>
+    <s v="Female"/>
+    <x v="17"/>
+    <x v="28"/>
+    <x v="0"/>
+    <x v="0"/>
+    <s v="D001"/>
+    <s v="Dr. Rao"/>
+    <n v="50"/>
+  </r>
+  <r>
+    <x v="29"/>
+    <s v="Dinesh"/>
+    <n v="22"/>
+    <s v="Male"/>
+    <x v="18"/>
+    <x v="29"/>
+    <x v="1"/>
+    <x v="0"/>
+    <s v="D005"/>
+    <s v="Dr. Reddy"/>
+    <n v="70"/>
+  </r>
+</pivotCacheRecords>
+</file>
+
+<file path=xl/pivotCache/pivotCacheRecords2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="30">
+  <r>
+    <s v="A10001"/>
+    <s v="Praveen"/>
+    <n v="28"/>
+    <s v="Male"/>
+    <s v="Hyderabad"/>
+    <d v="2026-04-30T00:00:00"/>
+    <x v="0"/>
+    <s v="Yes"/>
+    <s v="D001"/>
+    <s v="Dr. Rao"/>
+    <n v="50"/>
+    <s v="Normal"/>
+  </r>
+  <r>
+    <s v="A10002"/>
+    <s v="Dhanush"/>
+    <n v="22"/>
+    <s v="Male"/>
+    <s v="Hyderabad"/>
+    <d v="2026-05-01T00:00:00"/>
+    <x v="1"/>
+    <s v="Yes"/>
+    <s v="D005"/>
+    <s v="Dr. Reddy"/>
+    <n v="70"/>
+    <s v="Normal"/>
+  </r>
+  <r>
+    <s v="A10003"/>
+    <s v="Harpreet"/>
+    <n v="22"/>
+    <s v="Male"/>
+    <s v="Hyderabad"/>
+    <d v="2026-05-02T00:00:00"/>
+    <x v="2"/>
+    <s v="No"/>
+    <s v="D002"/>
+    <s v="Dr. Mehta"/>
+    <n v="40"/>
+    <s v="Normal"/>
+  </r>
+  <r>
+    <s v="A10004"/>
+    <s v="Sekhar"/>
+    <n v="19"/>
+    <s v="Male"/>
+    <s v="Hyderabad"/>
+    <d v="2026-05-03T00:00:00"/>
+    <x v="3"/>
+    <s v="No"/>
+    <s v="D004"/>
+    <s v="Dr. Sharma"/>
+    <n v="35"/>
+    <s v="Normal"/>
+  </r>
+  <r>
+    <s v="A10005"/>
+    <s v="Rangayya"/>
+    <n v="20"/>
+    <s v="Male"/>
+    <s v="Gudivada"/>
+    <d v="2026-05-04T00:00:00"/>
+    <x v="4"/>
+    <s v="Yes"/>
+    <s v="D003"/>
+    <s v="Dr. Kumar"/>
+    <n v="60"/>
+    <s v="Normal"/>
+  </r>
+  <r>
+    <s v="A10006"/>
+    <s v="Rangamma"/>
+    <n v="18"/>
+    <s v="Female"/>
+    <s v="Gudivada"/>
+    <d v="2026-05-05T00:00:00"/>
+    <x v="0"/>
+    <s v="Yes"/>
+    <s v="D001"/>
+    <s v="Dr. Rao"/>
+    <n v="50"/>
+    <s v="Normal"/>
+  </r>
+  <r>
+    <s v="A10007"/>
+    <s v="Mogalayya"/>
+    <n v="25"/>
+    <s v="Male"/>
+    <s v="Begumpet"/>
+    <d v="2026-05-06T00:00:00"/>
+    <x v="2"/>
+    <s v="Yes"/>
+    <s v="D002"/>
+    <s v="Dr. Mehta"/>
+    <n v="40"/>
+    <s v="Normal"/>
+  </r>
+  <r>
+    <s v="A10008"/>
+    <s v="Jangayya"/>
+    <n v="45"/>
+    <s v="Male"/>
+    <s v="Amaravathi"/>
+    <d v="2026-05-07T00:00:00"/>
+    <x v="0"/>
+    <s v="Yes"/>
+    <s v="D001"/>
+    <s v="Dr. Rao"/>
+    <n v="50"/>
+    <s v="Senior"/>
+  </r>
+  <r>
+    <s v="A10009"/>
+    <s v="Madhu"/>
+    <n v="22"/>
+    <s v="Male"/>
+    <s v="Godavari"/>
+    <d v="2026-05-08T00:00:00"/>
+    <x v="1"/>
+    <s v="Yes"/>
+    <s v="D005"/>
+    <s v="Dr. Reddy"/>
+    <n v="70"/>
+    <s v="Normal"/>
+  </r>
+  <r>
+    <s v="A10010"/>
+    <s v="Rudra"/>
+    <n v="28"/>
+    <s v="Male"/>
+    <s v="Konaseema"/>
+    <d v="2026-05-09T00:00:00"/>
+    <x v="2"/>
+    <s v="Yes"/>
+    <s v="D002"/>
+    <s v="Dr. Mehta"/>
+    <n v="40"/>
+    <s v="Normal"/>
+  </r>
+  <r>
+    <s v="A10011"/>
+    <s v="Mehar"/>
+    <n v="29"/>
+    <s v="Female"/>
+    <s v="Malakpet"/>
+    <d v="2026-05-10T00:00:00"/>
+    <x v="3"/>
+    <s v="Yes"/>
+    <s v="D004"/>
+    <s v="Dr. Sharma"/>
+    <n v="35"/>
+    <s v="Normal"/>
+  </r>
+  <r>
+    <s v="A10012"/>
+    <s v="mohan"/>
+    <n v="34"/>
+    <s v="Male"/>
+    <s v="Kondaput"/>
+    <d v="2026-05-11T00:00:00"/>
+    <x v="4"/>
+    <s v="Yes"/>
+    <s v="D003"/>
+    <s v="Dr. Kumar"/>
+    <n v="60"/>
+    <s v="Senior"/>
+  </r>
+  <r>
+    <s v="A10013"/>
+    <s v="Radhika"/>
+    <n v="22"/>
+    <s v="Female"/>
+    <s v="Hafeezpet"/>
+    <d v="2026-05-12T00:00:00"/>
+    <x v="0"/>
+    <s v="Yes"/>
+    <s v="D001"/>
+    <s v="Dr. Rao"/>
+    <n v="50"/>
+    <s v="Normal"/>
+  </r>
+  <r>
+    <s v="A10014"/>
+    <s v="Mounika"/>
+    <n v="30"/>
+    <s v="Female"/>
+    <s v="High tech city"/>
+    <d v="2026-05-13T00:00:00"/>
+    <x v="2"/>
+    <s v="Yes"/>
+    <s v="D002"/>
+    <s v="Dr. Mehta"/>
+    <n v="40"/>
+    <s v="Normal"/>
+  </r>
+  <r>
+    <s v="A10015"/>
+    <s v="Meghana"/>
+    <n v="20"/>
+    <s v="Female"/>
+    <s v="Kondapur"/>
+    <d v="2026-05-14T00:00:00"/>
+    <x v="0"/>
+    <s v="No"/>
+    <s v="D001"/>
+    <s v="Dr. Rao"/>
+    <n v="50"/>
+    <s v="Normal"/>
+  </r>
+  <r>
+    <s v="A10016"/>
+    <s v="Nagalaxmi"/>
+    <n v="20"/>
+    <s v="Female"/>
+    <s v="Nandigama"/>
+    <d v="2026-05-15T00:00:00"/>
+    <x v="1"/>
+    <s v="Yes"/>
+    <s v="D005"/>
+    <s v="Dr. Reddy"/>
+    <n v="70"/>
+    <s v="Normal"/>
+  </r>
+  <r>
+    <s v="A10017"/>
+    <s v="Manoj"/>
+    <n v="29"/>
+    <s v="Male"/>
+    <s v="Nandigama"/>
+    <d v="2026-05-16T00:00:00"/>
+    <x v="2"/>
+    <s v="No"/>
+    <s v="D002"/>
+    <s v="Dr. Mehta"/>
+    <n v="40"/>
+    <s v="Normal"/>
+  </r>
+  <r>
+    <s v="A10018"/>
+    <s v="Rekha"/>
+    <n v="29"/>
+    <s v="Female"/>
+    <s v="Kondapur"/>
+    <d v="2026-05-17T00:00:00"/>
+    <x v="3"/>
+    <s v="No"/>
+    <s v="D004"/>
+    <s v="Dr. Sharma"/>
+    <n v="35"/>
+    <s v="Normal"/>
+  </r>
+  <r>
+    <s v="A10019"/>
+    <s v="Happie"/>
+    <n v="20"/>
+    <s v="Female"/>
+    <s v="Malakpet"/>
+    <d v="2026-05-18T00:00:00"/>
+    <x v="4"/>
+    <s v="Yes"/>
+    <s v="D003"/>
+    <s v="Dr. Kumar"/>
+    <n v="60"/>
+    <s v="Normal"/>
+  </r>
+  <r>
+    <s v="A10020"/>
+    <s v="Nagarjuna"/>
+    <n v="29"/>
+    <s v="Male"/>
+    <s v="Singareni"/>
+    <d v="2026-05-19T00:00:00"/>
+    <x v="0"/>
+    <s v="No"/>
+    <s v="D001"/>
+    <s v="Dr. Rao"/>
+    <n v="50"/>
+    <s v="Normal"/>
+  </r>
+  <r>
+    <s v="A10021"/>
+    <s v="Sikhar"/>
+    <n v="28"/>
+    <s v="Male"/>
+    <s v="Rajkot"/>
+    <d v="2026-05-20T00:00:00"/>
+    <x v="2"/>
+    <s v="Yes"/>
+    <s v="D002"/>
+    <s v="Dr. Mehta"/>
+    <n v="40"/>
+    <s v="Normal"/>
+  </r>
+  <r>
+    <s v="A10022"/>
+    <s v="Dhawan"/>
+    <n v="45"/>
+    <s v="Male"/>
+    <s v="Bengalore"/>
+    <d v="2026-05-21T00:00:00"/>
+    <x v="0"/>
+    <s v="Yes"/>
+    <s v="D001"/>
+    <s v="Dr. Rao"/>
+    <n v="50"/>
+    <s v="Senior"/>
+  </r>
+  <r>
+    <s v="A10023"/>
+    <s v="Neelambari"/>
+    <n v="34"/>
+    <s v="Female"/>
+    <s v="Hyderabad"/>
+    <d v="2026-05-22T00:00:00"/>
+    <x v="1"/>
+    <s v="Yes"/>
+    <s v="D005"/>
+    <s v="Dr. Reddy"/>
+    <n v="70"/>
+    <s v="Senior"/>
+  </r>
+  <r>
+    <s v="A10024"/>
+    <s v="Aravind"/>
+    <n v="22"/>
+    <s v="Male"/>
+    <s v="Hyderabad"/>
+    <d v="2026-05-23T00:00:00"/>
+    <x v="2"/>
+    <s v="No"/>
+    <s v="D002"/>
+    <s v="Dr. Mehta"/>
+    <n v="40"/>
+    <s v="Normal"/>
+  </r>
+  <r>
+    <s v="A10025"/>
+    <s v="Meghana"/>
+    <n v="24"/>
+    <s v="Female"/>
+    <s v="Hyderabad"/>
+    <d v="2026-05-24T00:00:00"/>
+    <x v="3"/>
+    <s v="No"/>
+    <s v="D004"/>
+    <s v="Dr. Sharma"/>
+    <n v="35"/>
+    <s v="Normal"/>
+  </r>
+  <r>
+    <s v="A10026"/>
+    <s v="Simha"/>
+    <n v="34"/>
+    <s v="Male"/>
+    <s v="Godavari"/>
+    <d v="2026-05-25T00:00:00"/>
+    <x v="4"/>
+    <s v="Yes"/>
+    <s v="D003"/>
+    <s v="Dr. Kumar"/>
+    <n v="60"/>
+    <s v="Senior"/>
+  </r>
+  <r>
+    <s v="A10027"/>
+    <s v="Reddy"/>
+    <n v="23"/>
+    <s v="Male"/>
+    <s v="Vizag"/>
+    <d v="2026-05-26T00:00:00"/>
+    <x v="0"/>
+    <s v="Yes"/>
+    <s v="D001"/>
+    <s v="Dr. Rao"/>
+    <n v="50"/>
+    <s v="Normal"/>
+  </r>
+  <r>
+    <s v="A10028"/>
+    <s v="Klassen"/>
+    <n v="34"/>
+    <s v="Male"/>
+    <s v="Petrorius"/>
+    <d v="2026-05-27T00:00:00"/>
+    <x v="2"/>
+    <s v="Yes"/>
+    <s v="D002"/>
+    <s v="Dr. Mehta"/>
+    <n v="40"/>
+    <s v="Senior"/>
+  </r>
+  <r>
+    <s v="A10029"/>
+    <s v="Mouna"/>
+    <n v="28"/>
+    <s v="Female"/>
+    <s v="Nalgonda"/>
+    <d v="2026-05-28T00:00:00"/>
+    <x v="0"/>
+    <s v="Yes"/>
+    <s v="D001"/>
+    <s v="Dr. Rao"/>
+    <n v="50"/>
+    <s v="Normal"/>
+  </r>
+  <r>
+    <s v="A10030"/>
+    <s v="Dinesh"/>
+    <n v="22"/>
+    <s v="Male"/>
+    <s v="Chennai"/>
+    <d v="2026-05-29T00:00:00"/>
+    <x v="1"/>
+    <s v="Yes"/>
+    <s v="D005"/>
+    <s v="Dr. Reddy"/>
+    <n v="70"/>
+    <s v="Normal"/>
+  </r>
+</pivotCacheRecords>
+</file>
+
+<file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{7899311A-25B3-410E-8467-5C8249AFECAC}" name="PivotTable11" cacheId="47" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Departments">
+  <location ref="J29:K35" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="12">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="14" showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="6">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="4"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="6"/>
+  </rowFields>
+  <rowItems count="6">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Count of Senior category" fld="11" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{A7BE5781-FE3D-488E-BDD4-871511A12C32}" name="PivotTable9" cacheId="43" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="city">
+  <location ref="A29:D50" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="12">
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="20">
+        <item x="3"/>
+        <item x="2"/>
+        <item x="14"/>
+        <item x="18"/>
+        <item x="4"/>
+        <item x="1"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="0"/>
+        <item x="5"/>
+        <item x="10"/>
+        <item x="7"/>
+        <item x="6"/>
+        <item x="17"/>
+        <item x="11"/>
+        <item x="16"/>
+        <item x="13"/>
+        <item x="12"/>
+        <item x="15"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField numFmtId="14" showAll="0">
+      <items count="31">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item x="14"/>
+        <item x="15"/>
+        <item x="16"/>
+        <item x="17"/>
+        <item x="18"/>
+        <item x="19"/>
+        <item x="20"/>
+        <item x="21"/>
+        <item x="22"/>
+        <item x="23"/>
+        <item x="24"/>
+        <item x="25"/>
+        <item x="26"/>
+        <item x="27"/>
+        <item x="28"/>
+        <item x="29"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisCol" showAll="0">
+      <items count="3">
+        <item x="1"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="15">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="4"/>
+  </rowFields>
+  <rowItems count="20">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i>
+      <x v="10"/>
+    </i>
+    <i>
+      <x v="11"/>
+    </i>
+    <i>
+      <x v="12"/>
+    </i>
+    <i>
+      <x v="13"/>
+    </i>
+    <i>
+      <x v="14"/>
+    </i>
+    <i>
+      <x v="15"/>
+    </i>
+    <i>
+      <x v="16"/>
+    </i>
+    <i>
+      <x v="17"/>
+    </i>
+    <i>
+      <x v="18"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="7"/>
+  </colFields>
+  <colItems count="3">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Count of Patient ID" fld="0" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <formats count="4">
+    <format dxfId="27">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="21">
+      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="4" count="18">
+            <x v="1"/>
+            <x v="2"/>
+            <x v="3"/>
+            <x v="4"/>
+            <x v="5"/>
+            <x v="6"/>
+            <x v="7"/>
+            <x v="8"/>
+            <x v="9"/>
+            <x v="10"/>
+            <x v="11"/>
+            <x v="12"/>
+            <x v="13"/>
+            <x v="14"/>
+            <x v="15"/>
+            <x v="16"/>
+            <x v="17"/>
+            <x v="18"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="20">
+      <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="19">
+      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="4" count="1">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+  </formats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2545611B-B54F-469B-9ECF-480AF8DB93D2}" name="PivotTable8" cacheId="43" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Departments">
+  <location ref="J17:K21" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
+  <pivotFields count="12">
+    <pivotField axis="axisPage" dataField="1" showAll="0">
+      <items count="31">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item x="14"/>
+        <item x="15"/>
+        <item x="16"/>
+        <item x="17"/>
+        <item x="18"/>
+        <item x="19"/>
+        <item x="20"/>
+        <item x="21"/>
+        <item x="22"/>
+        <item x="23"/>
+        <item x="24"/>
+        <item x="25"/>
+        <item x="26"/>
+        <item x="27"/>
+        <item x="28"/>
+        <item x="29"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="14" showAll="0">
+      <items count="31">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item x="14"/>
+        <item x="15"/>
+        <item x="16"/>
+        <item x="17"/>
+        <item x="18"/>
+        <item x="19"/>
+        <item x="20"/>
+        <item x="21"/>
+        <item x="22"/>
+        <item x="23"/>
+        <item x="24"/>
+        <item x="25"/>
+        <item x="26"/>
+        <item x="27"/>
+        <item x="28"/>
+        <item x="29"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" showAll="0" measureFilter="1" sortType="descending">
+      <items count="6">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="4"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+      <autoSortScope>
+        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
+          <references count="1">
+            <reference field="4294967294" count="1" selected="0">
+              <x v="0"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </autoSortScope>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="15">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="6"/>
+  </rowFields>
+  <rowItems count="4">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <pageFields count="1">
+    <pageField fld="0" hier="-1"/>
+  </pageFields>
+  <dataFields count="1">
+    <dataField name="Count of Patient ID" fld="0" subtotal="count" baseField="0" baseItem="0" numFmtId="1"/>
+  </dataFields>
+  <formats count="1">
+    <format dxfId="32">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+  </formats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <filters count="1">
+    <filter fld="6" type="count" evalOrder="-1" id="1" iMeasureFld="0">
+      <autoFilter ref="A1">
+        <filterColumn colId="0">
+          <top10 val="3" filterVal="3"/>
+        </filterColumn>
+      </autoFilter>
+    </filter>
+  </filters>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{A39E4CB7-CABD-476D-8454-6F44A4A51055}" name="PivotTable7" cacheId="43" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Months">
+  <location ref="E17:F20" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="12">
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="14" showAll="0">
+      <items count="31">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item x="14"/>
+        <item x="15"/>
+        <item x="16"/>
+        <item x="17"/>
+        <item x="18"/>
+        <item x="19"/>
+        <item x="20"/>
+        <item x="21"/>
+        <item x="22"/>
+        <item x="23"/>
+        <item x="24"/>
+        <item x="25"/>
+        <item x="26"/>
+        <item x="27"/>
+        <item x="28"/>
+        <item x="29"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0" sortType="descending">
+      <items count="15">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item t="default"/>
+      </items>
+      <autoSortScope>
+        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
+          <references count="1">
+            <reference field="4294967294" count="1" selected="0">
+              <x v="0"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </autoSortScope>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="11"/>
+  </rowFields>
+  <rowItems count="3">
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Count of Patient ID" fld="0" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <formats count="4">
+    <format dxfId="54">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="43">
+      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="11" count="1">
+            <x v="4"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="41">
+      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="11" count="1">
+            <x v="5"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="40">
+      <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+  </formats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{1EAB66F5-F279-4206-ACF4-38F95C536C22}" name="PivotTable6" cacheId="43" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Departments">
+  <location ref="A17:B23" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="12">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="14" showAll="0">
+      <items count="31">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item x="14"/>
+        <item x="15"/>
+        <item x="16"/>
+        <item x="17"/>
+        <item x="18"/>
+        <item x="19"/>
+        <item x="20"/>
+        <item x="21"/>
+        <item x="22"/>
+        <item x="23"/>
+        <item x="24"/>
+        <item x="25"/>
+        <item x="26"/>
+        <item x="27"/>
+        <item x="28"/>
+        <item x="29"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="6">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="4"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="15">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="6"/>
+  </rowFields>
+  <rowItems count="6">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Average of Age" fld="2" subtotal="average" baseField="6" baseItem="2" numFmtId="164"/>
+  </dataFields>
+  <formats count="1">
+    <format dxfId="56">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+  </formats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{8724B165-76AE-43CA-8569-071C93A24F73}" name="PivotTable5" cacheId="43" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Departments">
+  <location ref="O4:T25" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="12">
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="20">
+        <item x="3"/>
+        <item x="2"/>
+        <item x="14"/>
+        <item x="18"/>
+        <item x="4"/>
+        <item x="1"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="0"/>
+        <item x="5"/>
+        <item x="10"/>
+        <item x="7"/>
+        <item x="6"/>
+        <item x="17"/>
+        <item x="11"/>
+        <item x="16"/>
+        <item x="13"/>
+        <item x="12"/>
+        <item x="15"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField numFmtId="14" showAll="0">
+      <items count="31">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item x="14"/>
+        <item x="15"/>
+        <item x="16"/>
+        <item x="17"/>
+        <item x="18"/>
+        <item x="19"/>
+        <item x="20"/>
+        <item x="21"/>
+        <item x="22"/>
+        <item x="23"/>
+        <item x="24"/>
+        <item x="25"/>
+        <item x="26"/>
+        <item x="27"/>
+        <item x="28"/>
+        <item x="29"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisCol" showAll="0">
+      <items count="6">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="4"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="15">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="4"/>
+  </rowFields>
+  <rowItems count="20">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i>
+      <x v="10"/>
+    </i>
+    <i>
+      <x v="11"/>
+    </i>
+    <i>
+      <x v="12"/>
+    </i>
+    <i>
+      <x v="13"/>
+    </i>
+    <i>
+      <x v="14"/>
+    </i>
+    <i>
+      <x v="15"/>
+    </i>
+    <i>
+      <x v="16"/>
+    </i>
+    <i>
+      <x v="17"/>
+    </i>
+    <i>
+      <x v="18"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="6"/>
+  </colFields>
+  <colItems count="5">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Count of Patient ID" fld="0" subtotal="count" baseField="6" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{85F8C5D4-17BA-4764-84B3-D8A5C553EA85}" name="PivotTable4" cacheId="43" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Departments">
+  <location ref="J4:L11" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="12">
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="14" showAll="0">
+      <items count="31">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item x="14"/>
+        <item x="15"/>
+        <item x="16"/>
+        <item x="17"/>
+        <item x="18"/>
+        <item x="19"/>
+        <item x="20"/>
+        <item x="21"/>
+        <item x="22"/>
+        <item x="23"/>
+        <item x="24"/>
+        <item x="25"/>
+        <item x="26"/>
+        <item x="27"/>
+        <item x="28"/>
+        <item x="29"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" showAll="0" sortType="descending">
+      <items count="6">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="4"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+      <autoSortScope>
+        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
+          <references count="2">
+            <reference field="4294967294" count="1" selected="0">
+              <x v="0"/>
+            </reference>
+            <reference field="7" count="1" selected="0">
+              <x v="1"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </autoSortScope>
+    </pivotField>
+    <pivotField axis="axisCol" showAll="0">
+      <items count="3">
+        <item x="1"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="15">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="6"/>
+  </rowFields>
+  <rowItems count="6">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="7"/>
+  </colFields>
+  <colItems count="2">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Count of Patient ID" fld="0" subtotal="count" showDataAs="percentOfTotal" baseField="6" baseItem="0" numFmtId="10"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable8.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{4161C22E-436C-4335-BD87-2F11710FA5D6}" name="PivotTable3" cacheId="43" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Departments">
+  <location ref="E4:G11" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="12">
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="14" showAll="0">
+      <items count="31">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item x="14"/>
+        <item x="15"/>
+        <item x="16"/>
+        <item x="17"/>
+        <item x="18"/>
+        <item x="19"/>
+        <item x="20"/>
+        <item x="21"/>
+        <item x="22"/>
+        <item x="23"/>
+        <item x="24"/>
+        <item x="25"/>
+        <item x="26"/>
+        <item x="27"/>
+        <item x="28"/>
+        <item x="29"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" showAll="0" sortType="descending">
+      <items count="6">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="4"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+      <autoSortScope>
+        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
+          <references count="2">
+            <reference field="4294967294" count="1" selected="0">
+              <x v="0"/>
+            </reference>
+            <reference field="7" count="1" selected="0">
+              <x v="1"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </autoSortScope>
+    </pivotField>
+    <pivotField axis="axisCol" showAll="0">
+      <items count="3">
+        <item x="1"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="15">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="6"/>
+  </rowFields>
+  <rowItems count="6">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="7"/>
+  </colFields>
+  <colItems count="2">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Count of Patient ID" fld="0" subtotal="count" showDataAs="percentOfTotal" baseField="6" baseItem="0" numFmtId="10"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable9.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{68D99AEC-82D0-49A6-B9DF-F4A5FB479A21}" name="PivotTable2" cacheId="43" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Departments">
+  <location ref="A4:B10" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="12">
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="14" showAll="0">
+      <items count="31">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item x="14"/>
+        <item x="15"/>
+        <item x="16"/>
+        <item x="17"/>
+        <item x="18"/>
+        <item x="19"/>
+        <item x="20"/>
+        <item x="21"/>
+        <item x="22"/>
+        <item x="23"/>
+        <item x="24"/>
+        <item x="25"/>
+        <item x="26"/>
+        <item x="27"/>
+        <item x="28"/>
+        <item x="29"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="6">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="4"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="15">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="6"/>
+  </rowFields>
+  <rowItems count="6">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Count of Patient ID" fld="0" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -798,7 +3461,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02135A4D-EFA1-4470-A892-777B228599E9}">
-  <dimension ref="A1:K31"/>
+  <dimension ref="A1:L31"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.33203125" bestFit="1" customWidth="1"/>
@@ -812,9 +3475,10 @@
     <col min="9" max="9" width="15" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="12.77734375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>29</v>
       </c>
@@ -848,8 +3512,11 @@
       <c r="K1" s="1" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L1" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>31</v>
       </c>
@@ -886,8 +3553,12 @@
         <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G2,Department_info!$A$2:$A$6,0))</f>
         <v>50</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L2" t="str">
+        <f>IF(C2&gt;30,"Senior","Normal")</f>
+        <v>Normal</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>33</v>
       </c>
@@ -924,8 +3595,12 @@
         <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G3,Department_info!$A$2:$A$6,0))</f>
         <v>70</v>
       </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L3" t="str">
+        <f t="shared" ref="L3:L31" si="0">IF(C3&gt;30,"Senior","Normal")</f>
+        <v>Normal</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>35</v>
       </c>
@@ -962,8 +3637,12 @@
         <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G4,Department_info!$A$2:$A$6,0))</f>
         <v>40</v>
       </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L4" t="str">
+        <f t="shared" si="0"/>
+        <v>Normal</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>37</v>
       </c>
@@ -1000,8 +3679,12 @@
         <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G5,Department_info!$A$2:$A$6,0))</f>
         <v>35</v>
       </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L5" t="str">
+        <f t="shared" si="0"/>
+        <v>Normal</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>39</v>
       </c>
@@ -1038,8 +3721,12 @@
         <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G6,Department_info!$A$2:$A$6,0))</f>
         <v>60</v>
       </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L6" t="str">
+        <f t="shared" si="0"/>
+        <v>Normal</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>41</v>
       </c>
@@ -1076,8 +3763,12 @@
         <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G7,Department_info!$A$2:$A$6,0))</f>
         <v>50</v>
       </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L7" t="str">
+        <f t="shared" si="0"/>
+        <v>Normal</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>43</v>
       </c>
@@ -1114,8 +3805,12 @@
         <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G8,Department_info!$A$2:$A$6,0))</f>
         <v>40</v>
       </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L8" t="str">
+        <f t="shared" si="0"/>
+        <v>Normal</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>45</v>
       </c>
@@ -1152,8 +3847,12 @@
         <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G9,Department_info!$A$2:$A$6,0))</f>
         <v>50</v>
       </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L9" t="str">
+        <f t="shared" si="0"/>
+        <v>Senior</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>47</v>
       </c>
@@ -1190,8 +3889,12 @@
         <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G10,Department_info!$A$2:$A$6,0))</f>
         <v>70</v>
       </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L10" t="str">
+        <f t="shared" si="0"/>
+        <v>Normal</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>49</v>
       </c>
@@ -1228,8 +3931,12 @@
         <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G11,Department_info!$A$2:$A$6,0))</f>
         <v>40</v>
       </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L11" t="str">
+        <f t="shared" si="0"/>
+        <v>Normal</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>51</v>
       </c>
@@ -1266,8 +3973,12 @@
         <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G12,Department_info!$A$2:$A$6,0))</f>
         <v>35</v>
       </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L12" t="str">
+        <f t="shared" si="0"/>
+        <v>Normal</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>53</v>
       </c>
@@ -1304,8 +4015,12 @@
         <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G13,Department_info!$A$2:$A$6,0))</f>
         <v>60</v>
       </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L13" t="str">
+        <f t="shared" si="0"/>
+        <v>Senior</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>55</v>
       </c>
@@ -1342,8 +4057,12 @@
         <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G14,Department_info!$A$2:$A$6,0))</f>
         <v>50</v>
       </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L14" t="str">
+        <f t="shared" si="0"/>
+        <v>Normal</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>57</v>
       </c>
@@ -1380,8 +4099,12 @@
         <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G15,Department_info!$A$2:$A$6,0))</f>
         <v>40</v>
       </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L15" t="str">
+        <f t="shared" si="0"/>
+        <v>Normal</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>59</v>
       </c>
@@ -1418,8 +4141,12 @@
         <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G16,Department_info!$A$2:$A$6,0))</f>
         <v>50</v>
       </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L16" t="str">
+        <f t="shared" si="0"/>
+        <v>Normal</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>61</v>
       </c>
@@ -1456,8 +4183,12 @@
         <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G17,Department_info!$A$2:$A$6,0))</f>
         <v>70</v>
       </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L17" t="str">
+        <f t="shared" si="0"/>
+        <v>Normal</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>63</v>
       </c>
@@ -1494,8 +4225,12 @@
         <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G18,Department_info!$A$2:$A$6,0))</f>
         <v>40</v>
       </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L18" t="str">
+        <f t="shared" si="0"/>
+        <v>Normal</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>65</v>
       </c>
@@ -1532,8 +4267,12 @@
         <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G19,Department_info!$A$2:$A$6,0))</f>
         <v>35</v>
       </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L19" t="str">
+        <f t="shared" si="0"/>
+        <v>Normal</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>67</v>
       </c>
@@ -1570,8 +4309,12 @@
         <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G20,Department_info!$A$2:$A$6,0))</f>
         <v>60</v>
       </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L20" t="str">
+        <f t="shared" si="0"/>
+        <v>Normal</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>69</v>
       </c>
@@ -1608,8 +4351,12 @@
         <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G21,Department_info!$A$2:$A$6,0))</f>
         <v>50</v>
       </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L21" t="str">
+        <f t="shared" si="0"/>
+        <v>Normal</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>71</v>
       </c>
@@ -1646,8 +4393,12 @@
         <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G22,Department_info!$A$2:$A$6,0))</f>
         <v>40</v>
       </c>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L22" t="str">
+        <f t="shared" si="0"/>
+        <v>Normal</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>73</v>
       </c>
@@ -1684,8 +4435,12 @@
         <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G23,Department_info!$A$2:$A$6,0))</f>
         <v>50</v>
       </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L23" t="str">
+        <f t="shared" si="0"/>
+        <v>Senior</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>75</v>
       </c>
@@ -1722,8 +4477,12 @@
         <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G24,Department_info!$A$2:$A$6,0))</f>
         <v>70</v>
       </c>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L24" t="str">
+        <f t="shared" si="0"/>
+        <v>Senior</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>77</v>
       </c>
@@ -1760,8 +4519,12 @@
         <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G25,Department_info!$A$2:$A$6,0))</f>
         <v>40</v>
       </c>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L25" t="str">
+        <f t="shared" si="0"/>
+        <v>Normal</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>79</v>
       </c>
@@ -1798,8 +4561,12 @@
         <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G26,Department_info!$A$2:$A$6,0))</f>
         <v>35</v>
       </c>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L26" t="str">
+        <f t="shared" si="0"/>
+        <v>Normal</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>80</v>
       </c>
@@ -1836,8 +4603,12 @@
         <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G27,Department_info!$A$2:$A$6,0))</f>
         <v>60</v>
       </c>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L27" t="str">
+        <f t="shared" si="0"/>
+        <v>Senior</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>82</v>
       </c>
@@ -1874,8 +4645,12 @@
         <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G28,Department_info!$A$2:$A$6,0))</f>
         <v>50</v>
       </c>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L28" t="str">
+        <f t="shared" si="0"/>
+        <v>Normal</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>84</v>
       </c>
@@ -1912,8 +4687,12 @@
         <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G29,Department_info!$A$2:$A$6,0))</f>
         <v>40</v>
       </c>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L29" t="str">
+        <f t="shared" si="0"/>
+        <v>Senior</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>86</v>
       </c>
@@ -1950,8 +4729,12 @@
         <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G30,Department_info!$A$2:$A$6,0))</f>
         <v>50</v>
       </c>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L30" t="str">
+        <f t="shared" si="0"/>
+        <v>Normal</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>88</v>
       </c>
@@ -1987,6 +4770,10 @@
       <c r="K31">
         <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G31,Department_info!$A$2:$A$6,0))</f>
         <v>70</v>
+      </c>
+      <c r="L31" t="str">
+        <f t="shared" si="0"/>
+        <v>Normal</v>
       </c>
     </row>
   </sheetData>
@@ -2207,4 +4994,917 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{901DD493-6832-4019-8BA5-A6C981183D21}">
+  <dimension ref="A4:T50"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="3.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.21875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.77734375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.21875" customWidth="1"/>
+    <col min="11" max="11" width="22.21875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="7" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="17.21875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11.21875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="9.109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="4" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A4" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="B4" t="s">
+        <v>116</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="J4" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="K4" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="O4" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="P4" s="7" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="5" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A5" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="B5" s="9">
+        <v>9</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="F5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G5" t="s">
+        <v>7</v>
+      </c>
+      <c r="J5" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="K5" t="s">
+        <v>8</v>
+      </c>
+      <c r="L5" t="s">
+        <v>7</v>
+      </c>
+      <c r="O5" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="P5" t="s">
+        <v>94</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>16</v>
+      </c>
+      <c r="R5" t="s">
+        <v>97</v>
+      </c>
+      <c r="S5" t="s">
+        <v>100</v>
+      </c>
+      <c r="T5" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="6" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A6" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" s="9">
+        <v>5</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="F6" s="10">
+        <v>6.6666666666666666E-2</v>
+      </c>
+      <c r="G6" s="10">
+        <v>0.23333333333333334</v>
+      </c>
+      <c r="J6" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="K6" s="10">
+        <v>6.6666666666666666E-2</v>
+      </c>
+      <c r="L6" s="10">
+        <v>0.23333333333333334</v>
+      </c>
+      <c r="O6" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="P6" s="9">
+        <v>1</v>
+      </c>
+      <c r="Q6" s="9"/>
+      <c r="R6" s="9"/>
+      <c r="S6" s="9"/>
+      <c r="T6" s="9"/>
+    </row>
+    <row r="7" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A7" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="B7" s="9">
+        <v>8</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F7" s="10">
+        <v>0</v>
+      </c>
+      <c r="G7" s="10">
+        <v>0.16666666666666666</v>
+      </c>
+      <c r="J7" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="K7" s="10">
+        <v>0</v>
+      </c>
+      <c r="L7" s="10">
+        <v>0.16666666666666666</v>
+      </c>
+      <c r="O7" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="P7" s="9"/>
+      <c r="Q7" s="9"/>
+      <c r="R7" s="9">
+        <v>1</v>
+      </c>
+      <c r="S7" s="9"/>
+      <c r="T7" s="9"/>
+    </row>
+    <row r="8" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A8" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="B8" s="9">
+        <v>4</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="F8" s="10">
+        <v>0.1</v>
+      </c>
+      <c r="G8" s="10">
+        <v>0.16666666666666666</v>
+      </c>
+      <c r="J8" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="K8" s="10">
+        <v>0.1</v>
+      </c>
+      <c r="L8" s="10">
+        <v>0.16666666666666666</v>
+      </c>
+      <c r="O8" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="P8" s="9">
+        <v>1</v>
+      </c>
+      <c r="Q8" s="9"/>
+      <c r="R8" s="9"/>
+      <c r="S8" s="9"/>
+      <c r="T8" s="9"/>
+    </row>
+    <row r="9" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A9" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="B9" s="9">
+        <v>4</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="F9" s="10">
+        <v>0</v>
+      </c>
+      <c r="G9" s="10">
+        <v>0.13333333333333333</v>
+      </c>
+      <c r="J9" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="K9" s="10">
+        <v>0</v>
+      </c>
+      <c r="L9" s="10">
+        <v>0.13333333333333333</v>
+      </c>
+      <c r="O9" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="P9" s="9"/>
+      <c r="Q9" s="9">
+        <v>1</v>
+      </c>
+      <c r="R9" s="9"/>
+      <c r="S9" s="9"/>
+      <c r="T9" s="9"/>
+    </row>
+    <row r="10" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A10" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="B10" s="9">
+        <v>30</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="F10" s="10">
+        <v>0.1</v>
+      </c>
+      <c r="G10" s="10">
+        <v>3.3333333333333333E-2</v>
+      </c>
+      <c r="J10" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="K10" s="10">
+        <v>0.1</v>
+      </c>
+      <c r="L10" s="10">
+        <v>3.3333333333333333E-2</v>
+      </c>
+      <c r="O10" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="P10" s="9"/>
+      <c r="Q10" s="9">
+        <v>1</v>
+      </c>
+      <c r="R10" s="9"/>
+      <c r="S10" s="9">
+        <v>1</v>
+      </c>
+      <c r="T10" s="9"/>
+    </row>
+    <row r="11" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="E11" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="F11" s="10">
+        <v>0.26666666666666666</v>
+      </c>
+      <c r="G11" s="10">
+        <v>0.73333333333333328</v>
+      </c>
+      <c r="J11" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="K11" s="10">
+        <v>0.26666666666666666</v>
+      </c>
+      <c r="L11" s="10">
+        <v>0.73333333333333328</v>
+      </c>
+      <c r="O11" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="P11" s="9">
+        <v>1</v>
+      </c>
+      <c r="Q11" s="9"/>
+      <c r="R11" s="9"/>
+      <c r="S11" s="9">
+        <v>1</v>
+      </c>
+      <c r="T11" s="9"/>
+    </row>
+    <row r="12" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="O12" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="P12" s="9">
+        <v>1</v>
+      </c>
+      <c r="Q12" s="9"/>
+      <c r="R12" s="9"/>
+      <c r="S12" s="9"/>
+      <c r="T12" s="9"/>
+    </row>
+    <row r="13" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="O13" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="P13" s="9"/>
+      <c r="Q13" s="9"/>
+      <c r="R13" s="9">
+        <v>1</v>
+      </c>
+      <c r="S13" s="9"/>
+      <c r="T13" s="9"/>
+    </row>
+    <row r="14" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="O14" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="P14" s="9">
+        <v>1</v>
+      </c>
+      <c r="Q14" s="9">
+        <v>2</v>
+      </c>
+      <c r="R14" s="9">
+        <v>2</v>
+      </c>
+      <c r="S14" s="9"/>
+      <c r="T14" s="9">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="J15" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="K15" t="s">
+        <v>117</v>
+      </c>
+      <c r="O15" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="P15" s="9"/>
+      <c r="Q15" s="9"/>
+      <c r="R15" s="9">
+        <v>1</v>
+      </c>
+      <c r="S15" s="9"/>
+      <c r="T15" s="9"/>
+    </row>
+    <row r="16" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="O16" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="P16" s="9">
+        <v>1</v>
+      </c>
+      <c r="Q16" s="9"/>
+      <c r="R16" s="9"/>
+      <c r="S16" s="9"/>
+      <c r="T16" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A17" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="B17" t="s">
+        <v>122</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="F17" t="s">
+        <v>116</v>
+      </c>
+      <c r="J17" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="K17" t="s">
+        <v>116</v>
+      </c>
+      <c r="O17" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="P17" s="9"/>
+      <c r="Q17" s="9"/>
+      <c r="R17" s="9"/>
+      <c r="S17" s="9">
+        <v>1</v>
+      </c>
+      <c r="T17" s="9"/>
+    </row>
+    <row r="18" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A18" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="B18" s="6">
+        <v>28.666666666666668</v>
+      </c>
+      <c r="E18" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="F18" s="11">
+        <v>29</v>
+      </c>
+      <c r="J18" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="K18" s="11">
+        <v>9</v>
+      </c>
+      <c r="O18" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="P18" s="9"/>
+      <c r="Q18" s="9"/>
+      <c r="R18" s="9"/>
+      <c r="S18" s="9">
+        <v>1</v>
+      </c>
+      <c r="T18" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A19" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B19" s="6">
+        <v>24</v>
+      </c>
+      <c r="E19" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="F19" s="11">
+        <v>1</v>
+      </c>
+      <c r="J19" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="K19" s="11">
+        <v>8</v>
+      </c>
+      <c r="O19" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="P19" s="9">
+        <v>1</v>
+      </c>
+      <c r="Q19" s="9"/>
+      <c r="R19" s="9"/>
+      <c r="S19" s="9"/>
+      <c r="T19" s="9"/>
+    </row>
+    <row r="20" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A20" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="B20" s="6">
+        <v>27.25</v>
+      </c>
+      <c r="E20" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="F20" s="11">
+        <v>30</v>
+      </c>
+      <c r="J20" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="K20" s="11">
+        <v>5</v>
+      </c>
+      <c r="O20" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="P20" s="9"/>
+      <c r="Q20" s="9">
+        <v>1</v>
+      </c>
+      <c r="R20" s="9">
+        <v>1</v>
+      </c>
+      <c r="S20" s="9"/>
+      <c r="T20" s="9"/>
+    </row>
+    <row r="21" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A21" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="B21" s="6">
+        <v>27</v>
+      </c>
+      <c r="J21" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="K21" s="11">
+        <v>22</v>
+      </c>
+      <c r="O21" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="P21" s="9"/>
+      <c r="Q21" s="9"/>
+      <c r="R21" s="9">
+        <v>1</v>
+      </c>
+      <c r="S21" s="9"/>
+      <c r="T21" s="9"/>
+    </row>
+    <row r="22" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A22" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="B22" s="6">
+        <v>25.25</v>
+      </c>
+      <c r="O22" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="P22" s="9"/>
+      <c r="Q22" s="9"/>
+      <c r="R22" s="9">
+        <v>1</v>
+      </c>
+      <c r="S22" s="9"/>
+      <c r="T22" s="9"/>
+    </row>
+    <row r="23" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A23" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="B23" s="6">
+        <v>26.833333333333332</v>
+      </c>
+      <c r="O23" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="P23" s="9">
+        <v>1</v>
+      </c>
+      <c r="Q23" s="9"/>
+      <c r="R23" s="9"/>
+      <c r="S23" s="9"/>
+      <c r="T23" s="9"/>
+    </row>
+    <row r="24" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="O24" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="P24" s="9">
+        <v>1</v>
+      </c>
+      <c r="Q24" s="9"/>
+      <c r="R24" s="9"/>
+      <c r="S24" s="9"/>
+      <c r="T24" s="9"/>
+    </row>
+    <row r="25" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="O25" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="P25" s="9">
+        <v>9</v>
+      </c>
+      <c r="Q25" s="9">
+        <v>5</v>
+      </c>
+      <c r="R25" s="9">
+        <v>8</v>
+      </c>
+      <c r="S25" s="9">
+        <v>4</v>
+      </c>
+      <c r="T25" s="9">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="29" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A29" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="B29" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="J29" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="K29" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="30" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A30" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="B30" t="s">
+        <v>8</v>
+      </c>
+      <c r="C30" t="s">
+        <v>7</v>
+      </c>
+      <c r="D30" t="s">
+        <v>115</v>
+      </c>
+      <c r="J30" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="K30" s="9">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A31" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B31" s="11"/>
+      <c r="C31" s="11">
+        <v>1</v>
+      </c>
+      <c r="D31" s="11">
+        <v>1</v>
+      </c>
+      <c r="J31" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="K31" s="9">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="32" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A32" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B32" s="11"/>
+      <c r="C32" s="11">
+        <v>1</v>
+      </c>
+      <c r="D32" s="11">
+        <v>1</v>
+      </c>
+      <c r="J32" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="K32" s="9">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A33" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="B33" s="11"/>
+      <c r="C33" s="11">
+        <v>1</v>
+      </c>
+      <c r="D33" s="11">
+        <v>1</v>
+      </c>
+      <c r="J33" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="K33" s="9">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A34" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B34" s="11"/>
+      <c r="C34" s="11">
+        <v>1</v>
+      </c>
+      <c r="D34" s="11">
+        <v>1</v>
+      </c>
+      <c r="J34" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="K34" s="9">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A35" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B35" s="11"/>
+      <c r="C35" s="11">
+        <v>2</v>
+      </c>
+      <c r="D35" s="11">
+        <v>2</v>
+      </c>
+      <c r="J35" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="K35" s="9">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A36" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B36" s="11"/>
+      <c r="C36" s="11">
+        <v>2</v>
+      </c>
+      <c r="D36" s="11">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A37" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="B37" s="11"/>
+      <c r="C37" s="11">
+        <v>1</v>
+      </c>
+      <c r="D37" s="11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A38" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="B38" s="11"/>
+      <c r="C38" s="11">
+        <v>1</v>
+      </c>
+      <c r="D38" s="11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A39" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B39" s="11">
+        <v>4</v>
+      </c>
+      <c r="C39" s="11">
+        <v>3</v>
+      </c>
+      <c r="D39" s="11">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A40" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B40" s="11"/>
+      <c r="C40" s="11">
+        <v>1</v>
+      </c>
+      <c r="D40" s="11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A41" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="B41" s="11">
+        <v>2</v>
+      </c>
+      <c r="C41" s="11"/>
+      <c r="D41" s="11">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A42" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="B42" s="11"/>
+      <c r="C42" s="11">
+        <v>1</v>
+      </c>
+      <c r="D42" s="11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A43" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B43" s="11"/>
+      <c r="C43" s="11">
+        <v>2</v>
+      </c>
+      <c r="D43" s="11">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A44" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="B44" s="11"/>
+      <c r="C44" s="11">
+        <v>1</v>
+      </c>
+      <c r="D44" s="11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A45" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B45" s="11">
+        <v>1</v>
+      </c>
+      <c r="C45" s="11">
+        <v>1</v>
+      </c>
+      <c r="D45" s="11">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A46" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B46" s="11"/>
+      <c r="C46" s="11">
+        <v>1</v>
+      </c>
+      <c r="D46" s="11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A47" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="B47" s="11"/>
+      <c r="C47" s="11">
+        <v>1</v>
+      </c>
+      <c r="D47" s="11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A48" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B48" s="11">
+        <v>1</v>
+      </c>
+      <c r="C48" s="11"/>
+      <c r="D48" s="11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A49" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="B49" s="11"/>
+      <c r="C49" s="11">
+        <v>1</v>
+      </c>
+      <c r="D49" s="11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A50" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="B50" s="11">
+        <v>8</v>
+      </c>
+      <c r="C50" s="11">
+        <v>22</v>
+      </c>
+      <c r="D50" s="11">
+        <v>30</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>